<commit_message>
hoan thanh frontend trang chu
</commit_message>
<xml_diff>
--- a/thuatngu.xlsx
+++ b/thuatngu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4863F66A-1BD4-41D8-9F9E-F3E9E1541B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBBB7DF-B572-4E6A-BB94-B6D92974E070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Thuat ngu hoc vu" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="133">
   <si>
     <t>OJT</t>
   </si>
@@ -46,39 +46,21 @@
     <t>Slot</t>
   </si>
   <si>
-    <t>1 ca học 90 phút</t>
-  </si>
-  <si>
     <t>Block</t>
   </si>
   <si>
-    <t>5-6 tuần học rồi thi</t>
-  </si>
-  <si>
     <t>Semester</t>
   </si>
   <si>
-    <t>Spring, Summer, Fall</t>
-  </si>
-  <si>
     <t>Credit</t>
   </si>
   <si>
-    <t>Tín chỉ</t>
-  </si>
-  <si>
     <t>Attendance</t>
   </si>
   <si>
-    <t>Điểm danh</t>
-  </si>
-  <si>
     <t>Assignment</t>
   </si>
   <si>
-    <t>Bài tập lớn</t>
-  </si>
-  <si>
     <t>Quiz</t>
   </si>
   <si>
@@ -88,9 +70,6 @@
     <t>Progress Test</t>
   </si>
   <si>
-    <t>Kiểm tra giữa kỳ</t>
-  </si>
-  <si>
     <t>Final Exam</t>
   </si>
   <si>
@@ -100,15 +79,9 @@
     <t>Average Mark</t>
   </si>
   <si>
-    <t>Điểm tổng kết</t>
-  </si>
-  <si>
     <t>GPA</t>
   </si>
   <si>
-    <t>Điểm trung bình tích lũy</t>
-  </si>
-  <si>
     <t>Transcript</t>
   </si>
   <si>
@@ -118,9 +91,6 @@
     <t>Retake</t>
   </si>
   <si>
-    <t>Học lại</t>
-  </si>
-  <si>
     <t>Improve Mark</t>
   </si>
   <si>
@@ -130,27 +100,15 @@
     <t>FAP</t>
   </si>
   <si>
-    <t>Lịch học, điểm, điểm danh, đơn từ</t>
-  </si>
-  <si>
     <t>LMS</t>
   </si>
   <si>
-    <t>Tài liệu học tập, assignment, quiz</t>
-  </si>
-  <si>
     <t>EOS</t>
   </si>
   <si>
-    <t>Thi trực tuyến</t>
-  </si>
-  <si>
     <t>FEID</t>
   </si>
   <si>
-    <t>Tài khoản sinh viên</t>
-  </si>
-  <si>
     <t>Email FPT</t>
   </si>
   <si>
@@ -163,15 +121,9 @@
     <t>kiểm tra cuối kì</t>
   </si>
   <si>
-    <t>điểm trung bình môn</t>
-  </si>
-  <si>
     <t>Wishlist</t>
   </si>
   <si>
-    <t>Đăng ký nguyện vọng mở lớp</t>
-  </si>
-  <si>
     <t>Prerequisite</t>
   </si>
   <si>
@@ -181,9 +133,6 @@
     <t>Drop Course</t>
   </si>
   <si>
-    <t>Hủy môn</t>
-  </si>
-  <si>
     <t>Học vượt</t>
   </si>
   <si>
@@ -199,15 +148,9 @@
     <t>TRS</t>
   </si>
   <si>
-    <t>Chương trình tiếng Anh dự bị</t>
-  </si>
-  <si>
     <t>LUK</t>
   </si>
   <si>
-    <t>Little UK - giao tiếp tiếng Anh</t>
-  </si>
-  <si>
     <t>Level</t>
   </si>
   <si>
@@ -217,12 +160,6 @@
     <t>Placement Test</t>
   </si>
   <si>
-    <t>Kiểm tra xếp lớp</t>
-  </si>
-  <si>
-    <t>Thực tập doanh nghiệp 3-4 tháng</t>
-  </si>
-  <si>
     <t>Đồ án tốt nghiệp nhóm</t>
   </si>
   <si>
@@ -241,9 +178,6 @@
     <t>Cóc Vàng</t>
   </si>
   <si>
-    <t>Danh hiệu sinh viên xuất sắc</t>
-  </si>
-  <si>
     <t>Vovinam</t>
   </si>
   <si>
@@ -253,9 +187,6 @@
     <t>Nhạc cụ dân tộc</t>
   </si>
   <si>
-    <t>Môn học đặc trưng</t>
-  </si>
-  <si>
     <t>PE</t>
   </si>
   <si>
@@ -268,51 +199,24 @@
     <t>Học phần/môn học</t>
   </si>
   <si>
-    <t>Môn tiên quyết phải học trước</t>
-  </si>
-  <si>
     <t>Corequisite</t>
   </si>
   <si>
-    <t>Môn học song hành</t>
-  </si>
-  <si>
-    <t>Học lại môn đã trượt hoặc muốn cải thiện điểm</t>
-  </si>
-  <si>
     <t>Improvement</t>
   </si>
   <si>
     <t>Học cải thiện điểm</t>
   </si>
   <si>
-    <t>Hệ thống quản lý học vụ của FPT</t>
-  </si>
-  <si>
-    <t>Hệ thống học tập trực tuyến</t>
-  </si>
-  <si>
-    <t>Hệ thống quản lý hoạt động sinh viên</t>
-  </si>
-  <si>
     <t>Academic Warning</t>
   </si>
   <si>
-    <t>Cảnh báo học vụ</t>
-  </si>
-  <si>
     <t>Probation</t>
   </si>
   <si>
-    <t>Tình trạng học tập cần theo dõi</t>
-  </si>
-  <si>
     <t>Suspend</t>
   </si>
   <si>
-    <t>Tạm dừng học do học vụ hoặc thủ tục</t>
-  </si>
-  <si>
     <t>Registration</t>
   </si>
   <si>
@@ -337,18 +241,12 @@
     <t>Định hướng chuyên sâu</t>
   </si>
   <si>
-    <t>On-the-Job Training - thực tập doanh nghiệp</t>
-  </si>
-  <si>
     <t>Capstone Project</t>
   </si>
   <si>
     <t>Workshop</t>
   </si>
   <si>
-    <t>Buổi chia sẻ chuyên đề</t>
-  </si>
-  <si>
     <t>Seminar</t>
   </si>
   <si>
@@ -364,9 +262,6 @@
     <t>Mentor</t>
   </si>
   <si>
-    <t>Người hướng dẫn học tập</t>
-  </si>
-  <si>
     <t>Lecturer</t>
   </si>
   <si>
@@ -386,9 +281,6 @@
   </si>
   <si>
     <t>Lab</t>
-  </si>
-  <si>
-    <t>Buổi thực hành</t>
   </si>
   <si>
     <t>Project</t>
@@ -506,6 +398,96 @@
 Kết nối với Giảng viên/Mentor: Giảng viên FPT phần lớn đều có kinh nghiệm thực chiến tại các doanh nghiệp. Đừng ngại hỏi họ về các case study thực tế hoặc xin lời khuyên về định hướng
 Laptop cá nhân, tài khoản trường, phần mềm yêu cầu của môn học, tài liệu tham khảo, lịch học và lịch nộp Assignment.
 Đi học đầy đủ để tránh thiếu điểm chuyên cần; Assignment và Project thường chiếm tỷ trọng lớn; không để dồn việc đến cuối Block.</t>
+  </si>
+  <si>
+    <t>Slot: Tiết học. Mỗi slot tại FPT thường kéo dài 90 phút.</t>
+  </si>
+  <si>
+    <t>Quãng thời gian học. Một học kỳ (Semester) tại FPT thường chia làm 2 Block nhỏ (mỗi block khoảng hơn 1 tháng) để học cuốn chiếu một số môn.</t>
+  </si>
+  <si>
+    <t>Học kỳ. Một năm học tại FPT có 3 học kỳ chính thức: Spring (Mùa Xuân), Summer (Mùa Hè), và Fall (Mùa Thu).</t>
+  </si>
+  <si>
+    <t>Tín chỉ. Đơn vị dùng để đo lường khối lượng học tập của một môn học.</t>
+  </si>
+  <si>
+    <t>Môn học / Khóa học cụ thể trong chương trình đào tạo.</t>
+  </si>
+  <si>
+    <t>Điểm trung bình của một môn học (được tính từ điểm thành phần theo tỷ lệ phần trăm quy định).</t>
+  </si>
+  <si>
+    <t>Điểm trung bình tích lũy của sinh viên (thường tính theo thang điểm 4.0 tại FPT).</t>
+  </si>
+  <si>
+    <t>Học lại. Sinh viên phải đóng tiền và học lại từ đầu môn đó do bị fail điểm thành phần hoặc vắng quá số buổi</t>
+  </si>
+  <si>
+    <t>Tính năng "Nguyện vọng" trên hệ thống, cho phép sinh viên chọn trước các môn mình muốn học ở kỳ tới để nhà trường sắp xếp lịch.</t>
+  </si>
+  <si>
+    <t>Hệ thống quản lý học vụ. Nơi xem lịch học, điểm danh, xem điểm, đóng học phí, gửi các dịch vụ một cửa..</t>
+  </si>
+  <si>
+    <t>Hệ thống quản lý học tập. Nơi nhận tài liệu, làm Quiz, nộp Assignment và xem link phòng học (nếu học online).</t>
+  </si>
+  <si>
+    <t>Hệ thống thi trực tuyến nội bộ của FPT, dùng để làm các bài thi trắc nghiệm cuối kỳ.</t>
+  </si>
+  <si>
+    <t>Tài khoản định danh của sinh viên thuộc tổ chức giáo dục FPT, dùng để đăng nhập một chạm vào các hệ thống.</t>
+  </si>
+  <si>
+    <t>Hủy môn học. Việc sinh viên xin rút không học môn đó nữa trong khung thời gian quy định trước khi kỳ học bắt đầu hoặc theo quy chế.</t>
+  </si>
+  <si>
+    <t>Nước Anh thu nhỏ. Không gian học tiếng Anh bắt buộc ở giai đoạn chuẩn bị, yêu cầu giao tiếp hoàn toàn bằng tiếng Anh.</t>
+  </si>
+  <si>
+    <t>Bài thi phân lớp đầu vào nhằm đánh giá trình độ tiếng Anh của tân sinh viên để xếp vào Level phù hợp.</t>
+  </si>
+  <si>
+    <t>Kỳ thực tập thực tế tại doanh nghiệp (thường vào học kỳ 6). Sinh viên làm việc như một nhân viên thực thụ.</t>
+  </si>
+  <si>
+    <t>Danh hiệu cao quý dành cho sinh viên có thành tích học tập và hoạt động phong trào xuất sắc nhất mỗi học kỳ của từng khối ngành.</t>
+  </si>
+  <si>
+    <t>Môn học nghệ thuật truyền thống bắt buộc (được chọn Đàn Tranh, Sáo, Nhị,</t>
+  </si>
+  <si>
+    <t>Buổi hội thảo ngắn, chia sẻ kiến thức thực tế hoặc kỹ năng mềm do trường hoặc doanh nghiệp tổ chức.</t>
+  </si>
+  <si>
+    <t>Phòng thực hành (phòng máy tính cấu hình cao hoặc phòng thí nghiệm chuyên dụng).</t>
+  </si>
+  <si>
+    <t>Người hướng dẫn, cố vấn (có thể là anh chị khóa trên, chuyên gia hoặc giảng viên hỗ trợ định hướng).</t>
+  </si>
+  <si>
+    <t>Môn tiên quyết. Môn học bắt buộc bạn phải đạt (Pass) thì mới được phép đăng ký học môn tiếp theo (Ví dụ: Phải pass CSD201 mới được học các môn nâng cao hơn).</t>
+  </si>
+  <si>
+    <t>Môn song hành. Môn học bắt buộc phải được đăng ký học cùng lúc với một môn học khác trong cùng một học kỳ.</t>
+  </si>
+  <si>
+    <t>Cảnh cáo học vụ. Áp dụng khi sinh viên có kết quả học tập quá kém hoặc vi phạm quy chế ở mức độ nhẹ.</t>
+  </si>
+  <si>
+    <t>Thử thách học vụ. Trạng thái báo động đỏ khi sinh viên bị cảnh cáo liên tiếp, nếu không cải thiện điểm số sẽ bị buộc thôi học.</t>
+  </si>
+  <si>
+    <t>: Đình chỉ học tập. Trạng thái sinh viên bị tạm dừng việc học tại trường trong một thời gian do vi phạm kỷ luật nghiêm trọng hoặc lý do đặc biệt.</t>
+  </si>
+  <si>
+    <t>huẩn tiếng Anh đầu ra hoặc các chương trình bổ trợ tiếng Anh theo chuẩn riêng của FPT.</t>
+  </si>
+  <si>
+    <t>Bài tập lớn / Đồ án môn học. Thường làm theo cá nhân hoặc nhóm và nộp theo tiến độ.</t>
+  </si>
+  <si>
+    <t>Bài kiểm tra tiến độ (kiểm tra giữa kỳ) để đánh giá quá trình học.</t>
   </si>
 </sst>
 </file>
@@ -872,7 +854,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="2" max="2" width="133" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -888,255 +870,255 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="B29" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
@@ -1144,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
@@ -1152,191 +1134,167 @@
         <v>1</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="B38" t="s">
-        <v>71</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B43" t="s">
-        <v>80</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>82</v>
+        <v>126</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>26</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B48" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B49" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>35</v>
-      </c>
-      <c r="B50" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>37</v>
-      </c>
-      <c r="B51" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="B52" t="s">
-        <v>90</v>
+        <v>127</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="B53" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="B54" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>95</v>
+        <v>63</v>
       </c>
       <c r="B55" t="s">
-        <v>96</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="B58" t="s">
-        <v>102</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
@@ -1344,12 +1302,12 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="B60" t="s">
         <v>2</v>
@@ -1357,90 +1315,90 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="B61" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="B62" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="B63" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>111</v>
+        <v>77</v>
       </c>
       <c r="B64" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
       <c r="B65" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="B66" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="B67" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="B68" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="B69" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>123</v>
+        <v>87</v>
       </c>
       <c r="B70" t="s">
-        <v>124</v>
+        <v>88</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1459,50 +1417,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>128</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>129</v>
+        <v>93</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>138</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>130</v>
+        <v>94</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>137</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>132</v>
+        <v>96</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>134</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>136</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cap nhat lai file thuatngu.xlsx moi tinh
</commit_message>
<xml_diff>
--- a/thuatngu.xlsx
+++ b/thuatngu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a15d8f22836db40c/Desktop/deadline/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A15D8F22836DB40C/Desktop/deadline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="14_{648E0658-3BF8-4494-A926-4B88B9FD542E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED6C4BA4-B7FC-4B24-B608-6615D4F19F5A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{469D3E8B-0801-411A-81FA-C96F6E57BB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -266,7 +266,218 @@
     <t xml:space="preserve">Attendance </t>
   </si>
   <si>
-    <t xml:space="preserve">Tại Đại học FPT, Attendance (Điểm danh) không chỉ là việc có mặt tại lớp, mà là một trong những "quy tắc vàng" sống còn quyết định việc bạn có được phép thi cuối kỳ hay không.
+    <t xml:space="preserve">Slot </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semester </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assignment </t>
+  </si>
+  <si>
+    <t>chậm kì</t>
+  </si>
+  <si>
+    <t>retake</t>
+  </si>
+  <si>
+    <t>1. Internship là gì?
+Internship (OJT - On the Job Training) là kỳ thực tập tại doanh nghiệp, một học kỳ bắt buộc tại Đại học FPT (thường kéo dài 4-8 tháng). Đây là giai đoạn sinh viên rời giảng đường để làm việc thực tế tại các công ty đối tác, nhằm tích lũy kinh nghiệm, kỹ năng nghề nghiệp và làm quen với môi trường làm việc chuyên nghiệp.
+2. Các quy định "Sống còn"
+•	Điều kiện tham gia: Sinh viên phải hoàn thành đủ số tín chỉ quy định (thường là sau khi kết thúc các kỳ học chuyên ngành cơ bản) và không bị nợ các môn tiên quyết quan trọng.
+•	Đơn vị thực tập: Bạn có thể tự tìm công ty (nếu thỏa mãn tiêu chuẩn nhà trường) hoặc ứng tuyển vào các doanh nghiệp nằm trong mạng lưới đối tác của Đại học FPT (thông qua bộ phận OJT của trường).
+•	Báo cáo thực tập: Trong quá trình thực tập, bạn phải hoàn thành các báo cáo định kỳ theo yêu cầu của cả giảng viên hướng dẫn tại trường và người quản lý tại doanh nghiệp.
+3. Hướng dẫn thực hiện chi tiết
+A. Chuẩn bị hồ sơ (Portfolio/CV)
+•	Cách làm: Xây dựng một CV chuyên nghiệp, highlight các dự án đã thực hiện tại các kỳ học trước. Hãy tận dụng những sản phẩm từ các bài Assignment để làm minh chứng năng lực.
+B. Quy trình đăng ký và kết nối
+•	Cách làm: Theo dõi thông tin trên hệ thống quản lý thực tập của trường hoặc cổng thông tin OJT.
+•	Lưu ý: Luôn cập nhật trạng thái của bạn trên hệ thống và tham gia đầy đủ các buổi định hướng (Orientation) do bộ phận OJT tổ chức.
+C. Trong kỳ thực tập
+•	Cách làm: Làm việc đúng giờ, tuân thủ nội quy công ty. Đặc biệt, hãy chủ động giữ liên lạc với giảng viên hướng dẫn tại trường (Academic Supervisor) để được hỗ trợ kịp thời nếu gặp khó khăn tại nơi làm việc.
+4. Lời khuyên "nằm lòng" để tối ưu hóa kỳ OJT
+•	Chọn công ty theo định hướng nghề nghiệp: Đừng chỉ chọn nơi nào "dễ". Hãy chọn nơi bạn có thể học được kỹ năng mình thiếu hoặc nơi bạn dự định làm việc sau khi ra trường.
+•	Xem OJT như một "phỏng vấn dài hạn": Nhiều sinh viên được nhận vào làm chính thức ngay sau khi kết thúc kỳ thực tập. Hãy thể hiện thái độ làm việc chuyên nghiệp, cầu thị và trách nhiệm.
+•	Ghi chép nhật ký công việc: Đừng đợi đến cuối kỳ mới ngồi viết báo cáo. Hãy ghi lại những gì mình học được, những vấn đề mình đã giải quyết mỗi tuần. Điều này giúp báo cáo thực tập của bạn trở nên sâu sắc và thuyết phục.
+•	Chủ động networking: Đừng chỉ ngồi làm việc một mình. Hãy kết nối với đồng nghiệp, người hướng dẫn (Mentor) tại công ty. Mối quan hệ trong kỳ thực tập là tài sản cực kỳ quý giá.
+5. Checklist kiểm tra nhanh
+•	[ ] Đã hoàn thành đủ tín chỉ điều kiện cho kỳ OJT chưa?
+•	[ ] CV/Portfolio đã được trau chuốt và phản ánh đúng năng lực hiện tại chưa?
+•	[ ] Đã nắm rõ các mốc deadline báo cáo thực tập (định kỳ) chưa?
+•	[ ] Đã có thông tin liên lạc của Giảng viên hướng dẫn tại trường chưa?
+Mẹo nhỏ: Trước khi bắt đầu, hãy tìm hiểu kỹ Rubric chấm điểm thực tập của trường. Bạn cần hiểu nhà trường đánh giá bạn dựa trên những tiêu chí nào (thái độ, kỹ năng, sản phẩm đầu ra...) để tập trung thể hiện đúng các điểm đó trong suốt kỳ thực tập.</t>
+  </si>
+  <si>
+    <t>phòng dịch vụ sinh viên</t>
+  </si>
+  <si>
+    <t>học phí</t>
+  </si>
+  <si>
+    <t>1. Tuition Fee là gì?
+Tuition Fee (Học phí) tại Đại học FPT là khoản chi phí sinh viên phải đóng để duy trì lộ trình học tập. ĐH FPT áp dụng mô hình thu học phí theo gói (tín chỉ) hoặc học kỳ, tùy thuộc vào hợp đồng đào tạo bạn đã ký lúc nhập học. Việc quản lý học phí chặt chẽ là điều kiện tiên quyết để bạn giữ trạng thái "Active" (đang học) trên hệ thống.
+2. Các khoản phí chính
+•	Học phí chính khóa: Tính theo tín chỉ hoặc mức cố định theo kỳ (tùy theo khóa và chương trình).
+•	Học phí tiếng Anh dự bị: Khoản phí bắt buộc nếu bạn chưa đủ điều kiện tiếng Anh đầu vào.
+•	Phí giáo trình: Thường đã bao gồm trong học phí hoặc được tính riêng tùy theo quy định của từng cơ sở.
+•	Phí môn học lại/học cải thiện: Phát sinh nếu bạn đăng ký Retake hoặc cải thiện điểm.
+3. Hướng dẫn thực hiện đóng học phí
+A. Tra cứu số tiền cần đóng
+•	Cách làm: Đăng nhập vào FAP -&gt; Chọn mục Financial -&gt; View tuition.
+•	Lưu ý: Hệ thống luôn cập nhật số dư, số tiền đã đóng và số tiền còn thiếu. Hãy kiểm tra định kỳ trước mỗi đợt hạn chót (Deadline).
+B. Quy trình thanh toán
+•	Cách làm: Thanh toán qua mã QR (trong FAP), chuyển khoản ngân hàng theo đúng Mã số sinh viên + Họ tên (theo quy định của từng cơ sở).
+•	Lưu ý: Sau khi chuyển khoản, hãy giữ lại biên lai/ảnh chụp giao dịch. Nếu sau 24-48h trạng thái trên FAP chưa cập nhật, hãy gửi biên lai đó cho Phòng Kế toán hoặc bộ phận hỗ trợ học phí.
+4. Lời khuyên "nằm lòng" để quản lý tài chính
+•	Luôn đóng sớm hơn Deadline: Đừng bao giờ để đến ngày cuối cùng mới đóng. Lỗi ngân hàng hoặc lỗi hệ thống vào giờ chót có thể khiến bạn bị trễ hạn, dẫn đến việc bị khóa quyền đăng ký môn học hoặc mất quyền thi.
+•	Lập kế hoạch tài chính: Nếu gia đình cần chuẩn bị tài chính, hãy chủ động xem trước mức học phí từng kỳ trong Hợp đồng đào tạo. Học phí tại FPT thường tăng nhẹ (tùy lộ trình) hoặc thay đổi dựa trên số tín chỉ bạn đăng ký, hãy dự phòng dư ra khoảng 5-10%.
+•	Tận dụng học bổng để giảm gánh nặng: Nếu GPA của bạn tốt, hãy săn các gói học bổng khuyến học để giảm bớt học phí. Đó là cách tốt nhất để "đầu tư" vào việc học.
+•	Liên hệ sớm nếu gặp khó khăn: Nếu gia đình gặp sự cố tài chính đột xuất, hãy chủ động viết đơn xin gia hạn học phí gửi lên Phòng Dịch vụ sinh viên trước ngày hết hạn. Đừng đợi đến khi bị khóa FAP mới xin, khả năng được duyệt sẽ thấp hơn rất nhiều.
+5. Checklist kiểm tra nhanh mỗi kỳ
+•	[ ] Đã check số tiền cần đóng trên FAP chưa?
+•	[ ] Đã nắm rõ hạn chót (Deadline) của đợt đóng học phí này chưa?
+•	[ ] Đã thanh toán và lưu lại ảnh biên lai chuyển khoản chưa?
+•	[ ] Trạng thái thanh toán trên FAP đã chuyển sang "Paid" (Đã thanh toán) chưa?
+Mẹo nhỏ: Hãy sử dụng tính năng "Reminder" trên điện thoại để đặt lịch nhắc đóng học phí trước deadline 3-5 ngày. Với sinh viên, việc bị khóa tài khoản chỉ vì quên đóng học phí là một trải nghiệm rất "đắt giá" và gây ảnh hưởng lớn đến tâm lý cũng như lộ trình học tập.</t>
+  </si>
+  <si>
+    <t>Final Grade</t>
+  </si>
+  <si>
+    <t>Course Schedule</t>
+  </si>
+  <si>
+    <t>IT Support</t>
+  </si>
+  <si>
+    <t>1. Feedback là gì?
+Feedback tại Đại học FPT là hoạt động bắt buộc và mang tính chất định kỳ nhằm giúp sinh viên đánh giá năng lực, phương pháp giảng dạy và thái độ của giảng viên. Đây là kênh thông tin quan trọng nhất để nhà trường nâng cao chất lượng đào tạo. Việc hoàn thành Feedback là điều kiện bắt buộc để bạn có thể xem điểm tổng kết môn học (Final Grade) trên FAP.
+2. Các cột mốc Feedback cần lưu ý
+•	Feedback giữa kỳ (Mid-term Feedback): Thường diễn ra sau khoảng 5-7 tuần học. Mục đích là để giảng viên nắm bắt tâm lý sinh viên, từ đó điều chỉnh tốc độ hoặc phương pháp giảng dạy ngay trong kỳ học đó.
+•	Feedback cuối kỳ (End-term Feedback): Diễn ra trước khi kết thúc học kỳ. Đây là bản đánh giá tổng quát về toàn bộ khóa học.
+•	Lưu ý: Nếu bạn không hoàn thành Feedback đúng hạn, hệ thống FAP sẽ tạm khóa tính năng xem điểm của môn học đó.
+3. Hướng dẫn thực hiện Feedback
+A. Cách thực hiện
+•	Cách làm: Truy cập FAP -&gt; Feedback -&gt; Feedback for lecturers.
+•	Lựa chọn: Hệ thống sẽ liệt kê danh sách các môn học và giảng viên tương ứng. Bạn chọn môn cần thực hiện và trả lời các câu hỏi đánh giá theo thang điểm (thường từ 1-5 hoặc 1-7).
+B. Quy trình bảo mật
+•	Lưu ý: Mọi đánh giá của bạn là ẩn danh. Giảng viên chỉ nhận được kết quả tổng hợp (điểm trung bình và các góp ý chung), họ không thể biết đích danh sinh viên nào đã viết ý kiến gì.
+4. Lời khuyên "nằm lòng" để Feedback có giá trị
+•	Tính trung thực: Đây là quyền lợi của bạn. Nếu phương pháp dạy quá nhanh, bài giảng khó hiểu, hay cách chấm điểm chưa hợp lý, hãy thẳng thắn góp ý. Ý kiến của bạn là cơ sở để nhà trường yêu cầu giảng viên cải thiện.
+•	Góp ý cụ thể (Phần comment): Đừng chỉ đánh giá bằng các con số. Ở phần bình luận, hãy ghi rõ các ví dụ cụ thể (ví dụ: "Giảng viên cần nói to hơn", "Nên cho thêm bài tập thực hành", "Tốc độ dạy hơi nhanh ở chương 3"). Những góp ý chi tiết này rất có giá trị với giảng viên.
+•	Tâm thế xây dựng: Feedback không phải là công cụ để "trả đũa" cá nhân. Hãy đánh giá công tâm dựa trên chất lượng môn học và thái độ của giảng viên. Một Feedback mang tính xây dựng sẽ được nhà trường và giảng viên coi trọng hơn nhiều.
+•	Đừng để đến phút cuối: Hãy hoàn thành Feedback ngay khi có thông báo. Đừng đợi đến đúng ngày xem điểm mới vào làm, lúc đó hệ thống có thể bị quá tải.
+5. Checklist kiểm tra nhanh
+•	[ ] Đã nhận được thông báo thực hiện Feedback trên FAP chưa?
+•	[ ] Đã hoàn thành Feedback cho tất cả các môn học trong kỳ chưa?
+•	[ ] Các góp ý đã được viết một cách cụ thể, rõ ràng chưa?
+•	[ ] Đã kiểm tra lại trên FAP xem môn học đó đã hiện trạng thái "Completed" (đã hoàn thành) chưa?
+Mẹo nhỏ: Hãy dành riêng 15 phút mỗi kỳ để thực hiện Feedback một cách nghiêm túc. Hãy coi đây là cách bạn góp phần định hình chất lượng đào tạo tại FPT. Một sinh viên biết cách Feedback văn minh và cụ thể cũng chính là người đang rèn luyện kỹ năng đánh giá (critical thinking) rất tốt cho công việc sau này.</t>
+  </si>
+  <si>
+    <t>1. Student Management là gì?
+Student Management (Quản lý sinh viên) tại Đại học FPT không phải là một chức năng đơn lẻ mà là một hệ thống các quy định, quy trình và bộ phận chuyên trách nhằm quản lý toàn diện đời sống, học tập và tư cách sinh viên từ khi nhập học đến khi tốt nghiệp. Hệ thống này đảm bảo mọi sinh viên tuân thủ đúng Quy chế đào tạo và Student Handbook.
+2. Các nhóm vấn đề trọng yếu
+•	Hồ sơ sinh viên: Quản lý thông tin cá nhân, bằng cấp đầu vào, giấy tờ lưu trữ.
+•	Trạng thái sinh viên (Status): Quản lý tình trạng học tập (Active, Bảo lưu - Suspend, Thôi học - Drop out, Tốt nghiệp).
+•	Điểm rèn luyện: Đánh giá đạo đức, sự tham gia phong trào, đóng góp cộng đồng.
+•	Kỷ luật học đường: Xử lý các vi phạm về quy chế thi cử, thái độ với giảng viên, hay các quy định về trang phục/tác phong tại trường.
+3. Hướng dẫn thực hiện các tác vụ liên quan
+A. Thủ tục hành chính (Bảo lưu, Chuyển cơ sở, Nghỉ học)
+•	Cách làm: Truy cập FAP -&gt; Student Service -&gt; Submit Request. Điền form và chờ xác nhận từ phòng quản lý sinh viên.
+•	Lưu ý: Mọi yêu cầu liên quan đến trạng thái học tập đều yêu cầu bạn phải có lý do chính đáng và kèm minh chứng (ví dụ: giấy khám bệnh, quyết định điều động công tác...).
+B. Theo dõi điểm rèn luyện
+•	Cách làm: Kiểm tra định kỳ tại mục Student Life trên FAP.
+•	Lưu ý: Điểm rèn luyện thấp có thể ảnh hưởng đến cơ hội xét học bổng và xét tốt nghiệp.
+C. Cập nhật thông tin cá nhân
+•	Cách làm: Luôn đảm bảo email cá nhân, số điện thoại, và địa chỉ liên lạc trên FAP là mới nhất. Đây là nguồn thông tin chính để nhà trường liên hệ với gia đình bạn trong các tình huống khẩn cấp.
+4. Lời khuyên "nằm lòng" để quản lý bản thân tốt nhất
+•	Hiểu rõ "Student Handbook": Đây là "bộ luật" của trường. Mọi hành vi của bạn nếu vi phạm sẽ bị xử lý theo quy định trong này. Hãy đọc ít nhất 1 lần để biết "đường biên" cho phép của mình đến đâu.
+•	Chủ động cập nhật trạng thái: Nếu bạn cần bảo lưu (vì lý do cá nhân hoặc tài chính), hãy làm đơn càng sớm càng tốt. Việc tự ý nghỉ học mà không làm thủ tục bảo lưu sẽ khiến bạn bị tính "vắng không phép" và dẫn đến bị buộc thôi học (Drop out).
+•	Xây dựng "Hồ sơ sạch": Trong suốt quá trình học, tránh để xảy ra các lỗi kỷ luật. Một hồ sơ kỷ luật không chỉ ảnh hưởng đến kỳ học đó mà còn có thể gây khó khăn khi bạn xin xác nhận thực tập hoặc xin việc sau này (một số doanh nghiệp sẽ yêu cầu xem bảng điểm rèn luyện/kỷ luật).
+•	Giữ liên hệ với "người quản lý trực tiếp": Biết được cán bộ nào phụ trách khối lớp của mình (Block Manager) là vô cùng quan trọng. Hãy lưu thông tin liên lạc của họ để hỏi ngay khi có thắc mắc về hồ sơ.
+5. Checklist kiểm tra nhanh
+•	[ ] Thông tin cá nhân (SĐT, Email) trên FAP đã chính xác chưa?
+•	[ ] Đã kiểm tra điểm rèn luyện định kỳ chưa? (Đủ điều kiện xét tốt nghiệp không?)
+•	[ ] Có đang dự định thay đổi trạng thái học tập (bảo lưu, chuyển cơ sở) không? Nếu có, đã tìm hiểu kỹ quy trình trên FAP chưa?
+•	[ ] Đã đọc quy chế về kỷ luật học đường chưa?
+Mẹo nhỏ: Hãy tạo một thư mục riêng trên máy tính hoặc Google Drive để lưu tất cả các văn bản, giấy xác nhận, biên lai học phí mà bạn đã làm thủ tục. Khi nhà trường cần kiểm tra lại hồ sơ quản lý của bạn, bạn có thể xuất trình bằng chứng ngay lập tức mà không mất thời gian chờ đợi tra cứu từ hệ thống.</t>
+  </si>
+  <si>
+    <t>Student Management</t>
+  </si>
+  <si>
+    <t>1. Project là gì?
+Tại Đại học FPT, Project là học phần thực hành quan trọng, nơi sinh viên vận dụng kiến thức lý thuyết đã học trong một hoặc nhiều môn chuyên ngành để xây dựng một sản phẩm thực tế (phần mềm, ứng dụng, website, nghiên cứu...). Đây là "bài thi tổng hợp" thay thế cho các kỳ thi truyền thống, giúp sinh viên làm quen với cách làm việc nhóm và quy trình phát triển sản phẩm chuyên nghiệp.
+2. Các quy định "Sống còn"
+•	Hình thức: Thường là làm theo nhóm (từ 3-5 thành viên).
+•	Quy trình chuẩn: Sinh viên phải thực hiện theo đúng các giai đoạn: Requirement Analysis (Phân tích) -&gt; Design (Thiết kế) -&gt; Implementation (Lập trình) -&gt; Testing (Kiểm thử) -&gt; Documentation (Viết báo cáo).
+•	Deadline: Project thường có các cột mốc kiểm tra (Milestones/Reviews) định kỳ. Nếu không hoàn thành đúng tiến độ từng Milestone, nhóm sẽ bị đánh giá thấp hoặc thậm chí là "cấm thi" bảo vệ cuối kỳ.
+3. Hướng dẫn thực hiện chi tiết
+A. Xây dựng nhóm
+•	Cách làm: Tìm các thành viên có kỹ năng bổ trợ cho nhau (ví dụ: người giỏi code, người giỏi tài liệu, người giỏi trình bày).
+•	Lưu ý: "Chọn bạn mà chơi" trong Project là yếu tố quyết định 70% thành bại. Hãy chọn những thành viên có trách nhiệm và cùng mục tiêu điểm số.
+B. Quản lý công việc (Work Management)
+•	Cách làm: Sử dụng các công cụ quản lý dự án như Trello, Jira, hoặc GitHub Projects. Phải có bảng phân chia công việc (Task) rõ ràng cho từng thành viên.
+•	Lưu ý: Mọi công việc phải được ghi nhận (Track). Đừng làm việc theo kiểu "ai tiện thì làm", sẽ dẫn đến tình trạng tranh chấp hoặc đùn đẩy trách nhiệm khi gần đến ngày nộp bài.
+C. Bảo vệ Project
+•	Cách làm: Chuẩn bị slide trình bày (Presentation) thật chuyên nghiệp, nắm vững kiến thức sản phẩm và có khả năng trả lời phản biện (Q&amp;A) từ giảng viên.
+4. Lời khuyên "nằm lòng" để đạt điểm cao
+•	Bám sát Rubric: Giảng viên chấm điểm dựa trên bộ tiêu chí (Rubric) đã ban hành. Hãy đọc kỹ nó trước khi bắt đầu. Nếu Rubric nhấn mạnh vào "Tính năng mới", hãy tập trung làm tính năng đó trước thay vì chỉ chăm chút giao diện.
+•	Documentation quan trọng không kém Code: Đừng coi nhẹ bài báo cáo (Documentation). Nhiều nhóm làm sản phẩm cực tốt nhưng báo cáo sơ sài dẫn đến điểm tổng kết rất thấp. Hãy trình bày tài liệu theo đúng form chuẩn của trường.
+•	Tận dụng giảng viên hướng dẫn (Mentor): Đừng đợi đến khi sản phẩm "tắt thở" mới hỏi giảng viên. Hãy chủ động cập nhật tiến độ (Meeting định kỳ) với Mentor để được chỉnh hướng ngay khi đi sai đường.
+•	Giải quyết xung đột nội bộ sớm: Nếu nhóm có thành viên không làm việc, hãy giải quyết ngay từ Milestone đầu tiên. Đừng đợi đến cuối kỳ mới báo cáo với giảng viên, lúc đó việc tách nhóm hay thay đổi nhân sự sẽ rất khó khăn.
+5. Checklist kiểm tra nhanh
+•	[ ] Đã hiểu rõ yêu cầu (Requirements) của đề bài chưa?
+•	[ ] Đã phân chia Task cho từng thành viên trên công cụ quản lý chưa?
+•	[ ] Đã có lịch họp nhóm định kỳ hàng tuần chưa?
+•	[ ] Đã nắm rõ các mốc Review/Milestone chưa?
+Mẹo nhỏ: Hãy dành thời gian làm Demo sớm. Sản phẩm chạy được sớm dù chỉ là bản thô (Prototype) sẽ giúp bạn nhận được phản hồi từ giảng viên ngay từ đầu. Điều này giúp bạn tránh phải "đập đi xây lại" toàn bộ dự án vào tuần cuối cùng trước ngày nộp bài.</t>
+  </si>
+  <si>
+    <t>Tại Đại học FPT, GPA (Grade Point Average) không chỉ là những con số trên bảng điểm; nó là "tấm hộ chiếu" quyết định học bổng, cơ hội thực tập, và quan trọng nhất là năng lực tốt nghiệp của bạn.
+Dưới đây là thông tin chi tiết nhất về GPA tại ĐH FPT.
+1. Phân biệt các loại GPA tại ĐH FPT
+Bạn cần nắm rõ 3 chỉ số này vì chúng phục vụ các mục đích hoàn toàn khác nhau:
+	Course Grade (Điểm tổng kết môn): Điểm số cuối cùng của từng môn học (thang điểm 10, quy đổi ra thang điểm chữ A, B, C, D, F).
+	Semester GPA (SGPA - Điểm trung bình học kỳ): Trung bình cộng có trọng số của các môn học trong duy nhất 1 học kỳ. Chỉ số này đánh giá phong độ học tập ngắn hạn của bạn.
+	Cumulative GPA (CGPA - Điểm trung bình tích lũy): Trung bình cộng của tất cả các môn học từ lúc nhập học đến thời điểm hiện tại. Đây là chỉ số quan trọng nhất.
+2. Cách tính GPA
+ĐH FPT quy đổi thang điểm 10 sang thang điểm 4 (hệ tín chỉ).
+Bảng quy đổi tham khảo:
+	A+ (9.0 - 10.0): 4.0
+	A (8.5 - 8.9): 3.75
+	A- (8.0 - 8.4): 3.5
+	B+ (7.5 - 7.9): 3.25
+	B (7.0 - 7.4): 3.0
+	C+ (6.5 - 6.9): 2.5
+	C (5.0 - 6.4): 2.0
+	F (Dưới 5.0): 0
+Công thức tính:
+GPA=(∑("Điểm chữ quy đổi" ×"Số tín chỉ" ) ) / (∑("Tổng số tín chỉ" ) )
+3. Hướng dẫn quản lý GPA
+Bước 1: Theo dõi chủ động
+	Đừng đợi đến khi nhà trường công bố. Hãy vào FAP -&gt; Report -&gt; Academic Transcript. Tại đây, hệ thống đã tính sẵn SGPA và CGPA cho bạn.
+	Nếu thấy điểm số không đúng với kết quả học tập (điểm thành phần bị sót), phải làm đơn khiếu nại ngay trong vòng 48 giờ kể từ khi công bố.
+Bước 2: Bảo vệ GPA
+	Điểm liệt (F): Một điểm F sẽ kéo tụt CGPA của bạn rất mạnh vì nó được tính là 0.0 điểm. Hãy ưu tiên học lại sớm để thay thế điểm 0 này bằng điểm số mới.
+	Cảnh báo học vụ (Academic Warning): Nếu CGPA rơi xuống dưới mức quy định (thường là dưới 2.0 hoặc 2.5 tùy khóa), bạn sẽ bị cảnh báo. Nếu không cải thiện trong các kỳ tiếp theo, bạn sẽ bị buộc thôi học.
+Bước 3: Tối ưu hóa GPA
+	Chọn môn thông minh: Khi đăng ký tín chỉ, hãy cân đối giữa môn nặng và môn nhẹ. Tránh việc dồn 3-4 môn nặng (coding, project) vào cùng một học kỳ nếu bạn không có sức bền.
+4. Lời khuyên "nằm lòng" từ chiến lược học tập
+	GPA 3.2+ là mục tiêu vàng: Với mức CGPA trên 3.2, bạn không chỉ dễ dàng đạt học bổng mà còn có lợi thế cực lớn khi ứng tuyển thực tập (OJT) tại các doanh nghiệp đối tác của FPT.
+	Đừng "nuôi" điểm F: Một điểm F không chỉ làm xấu bảng điểm mà còn gây áp lực tài chính (phải đóng học phí học lại) và áp lực thời gian (lộ trình học bị chậm lại). Hãy coi việc tránh điểm F là ưu tiên số 1, hơn cả việc cố đạt điểm A.
+	Tận dụng "Cải thiện điểm": Nếu bạn có một môn điểm C và muốn nâng GPA lên, hãy tìm hiểu quy định về học cải thiện (tùy thời điểm trường cho phép). Tuy nhiên, hãy cân nhắc kỹ về chi phí và thời gian.
+	Sử dụng công cụ giả lập: Hãy lập một bảng Google Sheets nhỏ. Cứ sau mỗi bài Assignment lớn, hãy điền điểm vào để tính toán xem mình cần bao nhiêu điểm ở bài Final để đạt được GPA mục tiêu của kỳ đó.
+5. Những câu hỏi cần tự vấn định kỳ (Checklist)
+	[ ] Mục tiêu của mình là gì? (Giữ học bổng, tránh cảnh báo, hay tốt nghiệp loại Giỏi?)
+	[ ] CGPA hiện tại có đang an toàn không? (Có cách xa ngưỡng cảnh báo học vụ không?)
+	[ ] Trong kỳ này, môn nào là "bom nổ chậm"? (Môn nào có khả năng kéo tụt GPA nhất?) -&gt; Dành thời gian tập trung vào môn đó trước.
+Lời khuyên đặc biệt:
+GPA tại ĐH FPT phản ánh tính cách của bạn: Sự kỷ luật và khả năng quản lý thời gian. Đừng nhìn vào con số để áp lực, hãy nhìn vào con số để điều chỉnh tốc độ học.</t>
+  </si>
+  <si>
+    <t>Tại Đại học FPT, Attendance (Điểm danh) không chỉ là việc có mặt tại lớp, mà là một trong những "quy tắc vàng" sống còn quyết định việc bạn có được phép thi cuối kỳ hay không.
 Dưới đây là thông tin chi tiết và cẩm nang quản lý Attendance dành cho sinh viên FPT.
 1. Định nghĩa &amp; Bản chất
 •	Attendance: Là số buổi bạn có mặt tại lớp (theo các Slot học).
@@ -279,7 +490,7 @@
 •	Điểm danh qua thiết bị: Một số môn học đặc thù có thể sử dụng các ứng dụng chuyên dụng để điểm danh theo thời gian thực.
 Cách kiểm soát Attendance:
 1.	Truy cập FAP: Đăng nhập vào FAP (FPT Academic Portal).
-2.	Mục Attendance: Chọn Attendance -&gt; View attendance để xem chi tiết số buổi đã vắng, buổi nào đã vắng và tình trạng hiện tại.
+2.	Mục Report: Chọn Attendance -&gt; View attendance để xem chi tiết số buổi đã vắng, buổi nào đã vắng và tình trạng hiện tại.
 3.	Đối soát: Sau mỗi buổi học, nếu bạn có mặt nhưng hệ thống lại ghi là vắng, hãy báo ngay với giảng viên trong vòng 24h - 48h. Nếu để quá lâu, giảng viên sẽ không thể can thiệp sửa đổi trên hệ thống.
 3. Những lưu ý "Sống còn" (Must-Know)
 •	Đừng xin giảng viên "cho em vắng thêm": Giảng viên không có quyền "xóa" buổi vắng cho bạn một cách tùy tiện vì hệ thống điểm danh được quản lý tập trung. Nếu bạn có lý do chính đáng (ốm đau, việc gia đình), bạn phải có minh chứng (giấy khám bệnh, đơn từ...) gửi cho Phòng Dịch vụ sinh viên (Service Center) hoặc Cố vấn học tập để được xem xét theo quy định.
@@ -292,17 +503,13 @@
 4.	Kiểm tra FAP định kỳ: Hãy tạo thói quen: mỗi sáng thứ Hai, mở FAP lên check mục Attendance. Đừng để đến cuối kỳ mới tá hỏa vì mình bị cấm thi.
 Bảng tóm tắt quản lý:
 Tình trạng	Giải pháp
-Vắng ít	Tự quản lý, đảm bảo không vượt quá ngưỡng trong Syllabus.
-Sai sót (Có mặt mà hệ thống ghi vắng)	Liên hệ giảng viên ngay trong 24-48h.
+Vắng ít		Tự quản lý, đảm bảo không vượt quá ngưỡng trong Syllabus.
+Sai sót (Có mặt mà hệ thống ghi vắng)      Liên hệ giảng viên ngay trong 24-48h.
 Vắng do lý do bất khả kháng	Liên hệ Cố vấn học tập/Phòng DV Sinh viên sớm nhất có thể.
-Đã chạm ngưỡng cấm thi	Liên hệ giảng viên/Cố vấn để nắm rõ tình trạng (thường là không cứu được).
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slot </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tại Đại học FPT, Slot là đơn vị thời gian chuẩn được sử dụng để phân bổ lịch học, lịch thi và các hoạt động học thuật. Hiểu rõ về "Slot" là cách nhanh nhất để bạn làm chủ thời gian biểu tại trường.
+Đã chạm ngưỡng cấm thi	Liên hệ giảng viên/Cố vấn để nắm rõ tình trạng (thường là không cứu được).</t>
+  </si>
+  <si>
+    <t>Tại Đại học FPT, Slot là đơn vị thời gian chuẩn được sử dụng để phân bổ lịch học, lịch thi và các hoạt động học thuật. Hiểu rõ về "Slot" là cách nhanh nhất để bạn làm chủ thời gian biểu tại trường.
 1. Định nghĩa &amp; Bản chất
 •	Slot là gì? Slot là đơn vị thời gian học tập cơ bản. Một buổi học (tín chỉ) tại FPT được tính bằng số Slot nhất định.
 •	Thời lượng: Tại Đại học FPT, 1 Slot thường kéo dài 90 phút (1 tiếng 30 phút).
@@ -310,14 +517,14 @@
 •	Phân bổ: Lịch học được sắp xếp theo khung giờ cố định từ sáng đến tối, từ thứ Hai đến thứ Bảy.
 2. Các thông tin chi tiết cần nắm vững
 •	Giờ Slot (Tham khảo):
-o	Slot 1: 07:30 - 09:00
-o	Slot 2: 09:10 - 10:40
-o	Slot 3: 10:50 - 12:20
-o	Slot 4: 12:50 - 14:20
-o	Slot 5: 14:30 - 16:00
-o	Slot 6: 16:10 - 17:40
-o	Slot 7: 17:50 - 19:20
-(Lưu ý: Thời gian cụ thể có thể chênh lệch tùy theo cơ sở và quy định của từng học kỳ, bạn cần tra cứu lịch trên FAP).
+Khung giờ Slot học chuẩn (Cơ sở Đà Nẵng):
+•	Slot 1	07:00 - 08:30
+•	Slot 2	08:45 - 10:15
+•	Slot 3	10:30 - 12:00
+•	Slot 4	12:30 - 14:00
+•	Slot 5	14:15 - 15:45
+•	Slot 6	16:00 - 17:30 
+•	(Lưu ý: Thời gian cụ thể có thể chênh lệch tùy theo cơ sở và quy định của từng học kỳ, bạn cần tra cứu lịch trên FAP).
 •	Attendance (Điểm danh theo Slot): Giảng viên thường điểm danh theo từng buổi học (thường là sau mỗi Slot hoặc theo buổi gồm nhiều Slot). Vắng mặt quá số Slot quy định trong môn học sẽ dẫn đến Cấm thi (Not allowed).
 3. Hướng dẫn thực hiện &amp; Quản lý
 •	Tra cứu lịch học (Schedule):
@@ -337,14 +544,10 @@
 Thời lượng 1 Slot	90 phút
 Cách tra cứu	FAP (Weekly Schedule)
 Hệ quả bỏ Slot	Ảnh hưởng Attendance -&gt; Nguy cơ Cấm thi
-Nguồn tin cậy	Email FPT
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semester </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tại Đại học FPT, Semester (Học kỳ) không chỉ đơn giản là một khoảng thời gian học tập, mà là một đơn vị quản lý học vụ chặt chẽ với nhịp độ rất nhanh. Việc nắm vững cách vận hành của Semester là chìa khóa để bạn không bị "ngợp" và đảm bảo lộ trình tốt nghiệp đúng hạn.
+Nguồn tin cậy	Email FPT</t>
+  </si>
+  <si>
+    <t>Tại Đại học FPT, Semester (Học kỳ) không chỉ đơn giản là một khoảng thời gian học tập, mà là một đơn vị quản lý học vụ chặt chẽ với nhịp độ rất nhanh. Việc nắm vững cách vận hành của Semester là chìa khóa để bạn không bị "ngợp" và đảm bảo lộ trình tốt nghiệp đúng hạn.
 1. Định nghĩa &amp; Bản chất
 •	Học kỳ (Semester): Một học kỳ tại ĐH FPT thường kéo dài khoảng 3 đến 4 tháng.
 •	Cấu trúc 3 kỳ/năm: ĐH FPT vận hành theo hệ thống Học kỳ luân phiên (thường là Spring, Summer, Fall). Điều này có nghĩa là bạn học liên tục gần như cả năm, không có kỳ nghỉ hè dài như các trường đại học truyền thống.
@@ -377,12 +580,8 @@
 Trước kỳ	Đăng ký đủ tín chỉ, nộp học phí, kiểm tra lộ trình.
 Tuần 1-2	Tải Syllabus, nắm rõ các mốc deadline của Assignment.
 Giữa kỳ	Check FAP xem điểm thành phần đã khớp chưa, kiểm tra số buổi vắng.
-Cuối kỳ	Ôn tập Final, chuẩn bị thiết bị thi, kiểm tra lịch thi chính thức.
-Sau kỳ	Check điểm tổng kết, làm thủ tục phúc khảo (nếu có).
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assignment </t>
+Cuối kỳ	  	Ôn tập Final, chuẩn bị thiết bị thi, kiểm tra lịch thi chính thức.
+Sau kỳ		Check điểm tổng kết, làm thủ tục phúc khảo (nếu có).</t>
   </si>
   <si>
     <t>Tại Đại học FPT, Assignment không chỉ đơn thuần là "bài tập về nhà". Nó là linh hồn của phương pháp học tập Project-based Learning (Học tập dựa trên dự án). Đây là nơi bạn biến lý thuyết từ sách vở thành sản phẩm thực tế.
@@ -403,7 +602,7 @@
 Lưu vết (Versioning): Sử dụng Git (nếu làm kỹ thuật) hoặc Google Drive (lịch sử chỉnh sửa) để tránh mất file.
 Kiểm tra tính trung thực: FPT áp dụng phần mềm kiểm tra đạo văn (Turnitin) và các công cụ phát hiện AI. Tuyệt đối không copy-paste toàn bộ từ nguồn ngoài hoặc dùng AI viết hộ mà không chỉnh sửa, bạn sẽ bị kỷ luật nặng.
 Bước 4: Nộp bài và Phỏng vấn (Submission &amp; Interview)
-Nộp bài: Đảm bảo nộp đúng định dạng (pdf, zip, link Github...) lên hệ thống FAP hoặc LMS đúng giờ.
+Nộp bài: Đảm bảo nộp đúng định dạng (pdf, zip, link Github...) lên hệ thống Edunext đúng giờ.
 Interview (Phỏng vấn): Rất nhiều môn đòi hỏi bạn phải giải trình về sản phẩm. Giảng viên sẽ hỏi để kiểm tra xem có thực sự là bạn làm không. Nếu bạn không trả lời được các câu hỏi về logic code hoặc nội dung bài làm, bạn sẽ bị nghi ngờ gian lận.
 3. Lời khuyên "nằm lòng" (Pro Tips)
 "Quy tắc 3 ngày": Đừng bao giờ bắt đầu bài tập trước deadline 3 ngày. Hãy bắt đầu ngay khi có đề. Việc phát sinh lỗi kỹ thuật (bug, lỗi định dạng) thường xảy ra vào phút cuối.
@@ -419,10 +618,7 @@
 [ ] Đã check lại Rubric một lần cuối để đảm bảo đủ ý chưa?</t>
   </si>
   <si>
-    <t>chậm kì</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tại Đại học FPT, khái niệm "chậm kỳ" (thường được gọi là chậm tiến độ học tập so với lộ trình chuẩn) là tình trạng sinh viên không thể hoàn thành chương trình học theo đúng khung thời gian dự kiến (thường là 3 năm hoặc 3.5 năm).
+    <t>Tại Đại học FPT, khái niệm "chậm kỳ" (thường được gọi là chậm tiến độ học tập so với lộ trình chuẩn) là tình trạng sinh viên không thể hoàn thành chương trình học theo đúng khung thời gian dự kiến (thường là 3 năm hoặc 3.5 năm).
 Dưới đây là thông tin chi tiết, hướng dẫn và lời khuyên để bạn kiểm soát lộ trình của mình.
 1. Bản chất của "Chậm kỳ" tại ĐH FPT
 •	Nguyên nhân:
@@ -436,7 +632,7 @@
 o	Áp lực học thuật: Các học kỳ cuối có thể bị dồn môn, gây quá tải.
 2. Hướng dẫn quản lý và thực hiện (Khi rơi vào diện chậm kỳ)
 Bước 1: Xác định tình trạng (Tự đánh giá)
-•	Kiểm tra Curriculum (Khung chương trình đào tạo) trên FAP.
+•	Kiểm tra Curriculum ở mục Reports (Khung chương trình đào tạo) trên FAP.
 •	So sánh danh sách các môn bạn đã qua với khung chương trình chuẩn.
 •	Xem xét các môn nợ đang vướng mắc: Môn đó có phải là môn tiên quyết không? Nếu không học được nó, bạn có bị chặn các môn sau không?
 Bước 2: Liên hệ Cố vấn học tập (Academic Advisor) - QUAN TRỌNG NHẤT
@@ -455,20 +651,19 @@
 4. Bảng kiểm tra lộ trình (Dành cho bạn)
 Nếu bạn đang...	Hành động cần thực hiện ngay
 Nợ 1 môn	Đưa vào Wishlist ngay, ưu tiên học lại vào kỳ tới.
-Nợ nhiều môn	Gặp cố vấn học tập lập lộ trình học lại chi tiết cho từng kỳ.
+Nợ nhiều môn		Gặp cố vấn học tập lập lộ trình học lại chi tiết cho từng kỳ.
 Bị Cấm thi nhiều lần	Xem xét lại cách quản lý thời gian/điểm danh hoặc xin bảo lưu nếu cần.
-Sắp tốt nghiệp mà vẫn nợ	Ưu tiên tối đa các môn chưa qua, bỏ qua các môn tự chọn không bắt buộc để dồn sức.
-</t>
+Sắp tốt nghiệp mà vẫn nợ	Ưu tiên tối đa các môn chưa qua, bỏ qua các môn tự chọn không bắt buộc để dồn sức.</t>
   </si>
   <si>
     <t>Tại Đại học FPT, FAP (FPT Academic Portal) là "trái tim" quản lý mọi hoạt động của sinh viên. Nếu bạn không nắm vững FAP, việc học tập tại đây sẽ trở nên vô cùng khó khăn. Dưới đây là cẩm nang chi tiết nhất về hệ thống này.
 1. FAP là gì?
 FAP (FPT Academic Portal) là cổng thông tin học vụ dành riêng cho sinh viên FPT. Đây là nơi duy nhất bạn dùng để tra cứu lịch học, xem điểm, theo dõi tiến độ (Attendance), đăng ký môn học và thực hiện các thủ tục hành chính.
-2. Các chức năng "Sống còn" trên FAP
+2. Các chức năng  trên FAP
 Chức năng	Mục đích
 Weekly Schedule	Xem lịch học hàng tuần (Giờ, phòng, giảng viên, link học online).
 Attendance	Theo dõi số buổi vắng. Đây là nơi kiểm soát "tử huyệt" của bạn.
-Grade	Xem điểm thành phần, điểm tổng kết và GPA tích lũy.
+Mark Reports	Xem điểm thành phần, điểm tổng kết và GPA tích lũy.
 Curriculum	Xem lộ trình học tập, các môn tiên quyết.
 Register Wishlist	Đăng ký môn học lại (Fail/Not allowed).
 View Exam Schedule	Xem lịch thi cuối kỳ.
@@ -480,7 +675,7 @@
 •	Cách làm: Vào Attendance -&gt; View attendance.
 •	Mẹo: Đừng đợi đến cuối kỳ. Hãy kiểm tra mục này sau mỗi buổi học. Nếu bạn có đi học mà hệ thống ghi "Absent" (Vắng), bạn chỉ có 48 giờ để email cho giảng viên yêu cầu sửa. Sau thời gian này, dữ liệu thường được khóa.
 C. Theo dõi điểm số (Grade)
-•	Cách làm: Vào Grade -&gt; Academic Transcript.
+•	Cách làm: Vào Reports -&gt; Academic Transcript.
 •	Mẹo: Luôn đối chiếu điểm trên FAP với điểm giảng viên đã công bố tại lớp. Nếu có sai sót về nhập liệu, phải phản hồi ngay.
 D. Đăng ký môn học (Registration)
 •	Trong các đợt đăng ký, hệ thống sẽ mở các khung giờ. Bạn cần thao tác nhanh vì các môn "hot" thường hết slot chỉ trong vài phút.
@@ -500,10 +695,7 @@
 Mẹo nhỏ: FAP có một danh sách các "thủ tục hành chính" (như xin giấy xác nhận sinh viên, chuyển cơ sở...). Hãy khám phá các tab này sớm, vì đến khi cần gấp mà không biết tìm ở đâu sẽ rất mất thời gian.</t>
   </si>
   <si>
-    <t>retake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Retake là gì?
+    <t>1. Retake là gì?
 Retake (Học lại) là việc sinh viên đăng ký học lại một học phần đã bị Fail (F) hoặc Cấm thi (Not allowed) ở lần học trước đó. Đây là quy trình bắt buộc để sinh viên hoàn thành đủ số tín chỉ yêu cầu trong khung chương trình đào tạo để đủ điều kiện tốt nghiệp.
 2. Các trường hợp bắt buộc phải Retake
 •	Điểm tổng kết (Course Grade) &lt; 5.0 (thang 10): Điểm F.
@@ -526,53 +718,10 @@
 •	[ ] Đã xác định rõ môn nào bị F/Not allowed trên FAP chưa?
 •	[ ] Môn đó có phải là môn tiên quyết cho các môn kỳ sau không?
 •	[ ] Đã kiểm tra lịch mở lớp hoặc đăng ký Wishlist chưa?
-•	[ ] Đã chuẩn bị tài chính cho kỳ đóng học phí môn học lại chưa?
-</t>
-  </si>
-  <si>
-    <t>Tại Đại học FPT, GPA (Grade Point Average) không chỉ là những con số trên bảng điểm; nó là "tấm hộ chiếu" quyết định học bổng, cơ hội thực tập, và quan trọng nhất là năng lực tốt nghiệp của bạn.
-Dưới đây là thông tin chi tiết nhất về GPA tại ĐH FPT.
-1. Phân biệt các loại GPA tại ĐH FPT
-Bạn cần nắm rõ 3 chỉ số này vì chúng phục vụ các mục đích hoàn toàn khác nhau:
-	Course Grade (Điểm tổng kết môn): Điểm số cuối cùng của từng môn học (thang điểm 10, quy đổi ra thang điểm chữ A, B, C, D, F).
-	Semester GPA (SGPA - Điểm trung bình học kỳ): Trung bình cộng có trọng số của các môn học trong duy nhất 1 học kỳ. Chỉ số này đánh giá phong độ học tập ngắn hạn của bạn.
-	Cumulative GPA (CGPA - Điểm trung bình tích lũy): Trung bình cộng của tất cả các môn học từ lúc nhập học đến thời điểm hiện tại. Đây là chỉ số quan trọng nhất.
-2. Cách tính GPA
-ĐH FPT quy đổi thang điểm 10 sang thang điểm 4 (hệ tín chỉ).
-Bảng quy đổi tham khảo:
-	A+ (9.0 - 10.0): 4.0
-	A (8.5 - 8.9): 3.75
-	A- (8.0 - 8.4): 3.5
-	B+ (7.5 - 7.9): 3.25
-	B (7.0 - 7.4): 3.0
-	C+ (6.5 - 6.9): 2.5
-	C (5.0 - 6.4): 2.0
-	F (Dưới 5.0): 0
-Công thức tính:
-GPA=(∑("Điểm chữ quy đổi" ×"Số tín chỉ" ) ) / (∑("Tổng số tín chỉ" ) )
-3. Hướng dẫn quản lý GPA
-Bước 1: Theo dõi chủ động
-	Đừng đợi đến khi nhà trường công bố. Hãy vào FAP -&gt; Grade -&gt; Academic Transcript. Tại đây, hệ thống đã tính sẵn SGPA và CGPA cho bạn.
-	Nếu thấy điểm số không đúng với kết quả học tập (điểm thành phần bị sót), phải làm đơn khiếu nại ngay trong vòng 48 giờ kể từ khi công bố.
-Bước 2: Bảo vệ GPA
-	Điểm liệt (F): Một điểm F sẽ kéo tụt CGPA của bạn rất mạnh vì nó được tính là 0.0 điểm. Hãy ưu tiên học lại sớm để thay thế điểm 0 này bằng điểm số mới.
-	Cảnh báo học vụ (Academic Warning): Nếu CGPA rơi xuống dưới mức quy định (thường là dưới 2.0 hoặc 2.5 tùy khóa), bạn sẽ bị cảnh báo. Nếu không cải thiện trong các kỳ tiếp theo, bạn sẽ bị buộc thôi học.
-Bước 3: Tối ưu hóa GPA
-	Chọn môn thông minh: Khi đăng ký tín chỉ, hãy cân đối giữa môn nặng và môn nhẹ. Tránh việc dồn 3-4 môn nặng (coding, project) vào cùng một học kỳ nếu bạn không có sức bền.
-4. Lời khuyên "nằm lòng" từ chiến lược học tập
-	GPA 3.2+ là mục tiêu vàng: Với mức CGPA trên 3.2, bạn không chỉ dễ dàng đạt học bổng mà còn có lợi thế cực lớn khi ứng tuyển thực tập (OJT) tại các doanh nghiệp đối tác của FPT.
-	Đừng "nuôi" điểm F: Một điểm F không chỉ làm xấu bảng điểm mà còn gây áp lực tài chính (phải đóng học phí học lại) và áp lực thời gian (lộ trình học bị chậm lại). Hãy coi việc tránh điểm F là ưu tiên số 1, hơn cả việc cố đạt điểm A.
-	Tận dụng "Cải thiện điểm": Nếu bạn có một môn điểm C và muốn nâng GPA lên, hãy tìm hiểu quy định về học cải thiện (tùy thời điểm trường cho phép). Tuy nhiên, hãy cân nhắc kỹ về chi phí và thời gian.
-	Sử dụng công cụ giả lập: Hãy lập một bảng Google Sheets nhỏ. Cứ sau mỗi bài Assignment lớn, hãy điền điểm vào để tính toán xem mình cần bao nhiêu điểm ở bài Final để đạt được GPA mục tiêu của kỳ đó.
-5. Những câu hỏi cần tự vấn định kỳ (Checklist)
-	[ ] Mục tiêu của mình là gì? (Giữ học bổng, tránh cảnh báo, hay tốt nghiệp loại Giỏi?)
-	[ ] CGPA hiện tại có đang an toàn không? (Có cách xa ngưỡng cảnh báo học vụ không?)
-	[ ] Trong kỳ này, môn nào là "bom nổ chậm"? (Môn nào có khả năng kéo tụt GPA nhất?) -&gt; Dành thời gian tập trung vào môn đó trước.
-Lời khuyên đặc biệt:
-GPA tại ĐH FPT phản ánh tính cách của bạn: Sự kỷ luật và khả năng quản lý thời gian. Đừng nhìn vào con số để áp lực, hãy nhìn vào con số để điều chỉnh tốc độ học.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Average Mark là gì?
+•	[ ] Đã chuẩn bị tài chính cho kỳ đóng học phí môn học lại chưa?</t>
+  </si>
+  <si>
+    <t>1. Average Mark là gì?
 Average Mark tại Đại học FPT là điểm số trung bình của một môn học, được tổng hợp từ nhiều thành phần điểm khác nhau (thay vì chỉ dựa vào một kỳ thi cuối kỳ). Hệ thống này nhằm đánh giá toàn diện quá trình nỗ lực và năng lực thực tế của sinh viên trong suốt học kỳ.
 2. Cách tính Average Mark
 Điểm môn học thường được tính dựa trên tỷ trọng (weight) của các cột điểm thành phần trong Syllabus của môn đó:
@@ -582,7 +731,7 @@
 	Quy đổi: Kết quả cuối cùng sẽ được quy đổi ra thang điểm 10, sau đó quy đổi tiếp sang thang điểm chữ (A, B, C, D, F) để tính GPA.
 3. Hướng dẫn theo dõi và thực hiện
 A. Theo dõi điểm số chủ động
-	Cách làm: Vào menu Grade -&gt; Academic Transcript trên FAP.
+	Cách làm: Vào menu Reports -&gt; Academic Transcript trên FAP.
 	Lưu ý: Mọi điểm thành phần (Quiz, Assignment) sau khi giảng viên chấm xong đều sẽ được cập nhật lên hệ thống. Hãy kiểm tra thường xuyên để đảm bảo điểm của bạn đã được nhập đúng.
 B. Xử lý khi có sai sót
 	Cách làm: Nếu điểm hiển thị trên FAP không khớp với điểm giảng viên công bố, bạn cần liên hệ giảng viên ngay trong vòng 48 giờ.
@@ -597,41 +746,10 @@
 	[ ] Đã kiểm tra điểm thành phần (Quiz, Assignment) trên FAP ngay sau khi có kết quả chưa?
 	[ ] Có cột điểm nào bị thiếu hoặc ghi nhận sai không?
 	[ ] Đã tính toán thử xem mình cần bao nhiêu điểm ở bài Final để đạt mục tiêu môn học chưa?
-Mẹo nhỏ: Hãy lập một file Excel cá nhân để tự tính toán điểm môn học theo thời gian thực (real-time). Khi biết rõ mình đang đứng ở mức nào, bạn sẽ biết cần dồn bao nhiêu sức lực cho bài thi cuối kỳ để đạt được mức điểm mong muốn (ví dụ: đạt điểm B hoặc A).
-</t>
-  </si>
-  <si>
-    <t>1. Internship là gì?
-Internship (OJT - On the Job Training) là kỳ thực tập tại doanh nghiệp, một học kỳ bắt buộc tại Đại học FPT (thường kéo dài 4-8 tháng). Đây là giai đoạn sinh viên rời giảng đường để làm việc thực tế tại các công ty đối tác, nhằm tích lũy kinh nghiệm, kỹ năng nghề nghiệp và làm quen với môi trường làm việc chuyên nghiệp.
-2. Các quy định "Sống còn"
-•	Điều kiện tham gia: Sinh viên phải hoàn thành đủ số tín chỉ quy định (thường là sau khi kết thúc các kỳ học chuyên ngành cơ bản) và không bị nợ các môn tiên quyết quan trọng.
-•	Đơn vị thực tập: Bạn có thể tự tìm công ty (nếu thỏa mãn tiêu chuẩn nhà trường) hoặc ứng tuyển vào các doanh nghiệp nằm trong mạng lưới đối tác của Đại học FPT (thông qua bộ phận OJT của trường).
-•	Báo cáo thực tập: Trong quá trình thực tập, bạn phải hoàn thành các báo cáo định kỳ theo yêu cầu của cả giảng viên hướng dẫn tại trường và người quản lý tại doanh nghiệp.
-3. Hướng dẫn thực hiện chi tiết
-A. Chuẩn bị hồ sơ (Portfolio/CV)
-•	Cách làm: Xây dựng một CV chuyên nghiệp, highlight các dự án đã thực hiện tại các kỳ học trước. Hãy tận dụng những sản phẩm từ các bài Assignment để làm minh chứng năng lực.
-B. Quy trình đăng ký và kết nối
-•	Cách làm: Theo dõi thông tin trên hệ thống quản lý thực tập của trường hoặc cổng thông tin OJT.
-•	Lưu ý: Luôn cập nhật trạng thái của bạn trên hệ thống và tham gia đầy đủ các buổi định hướng (Orientation) do bộ phận OJT tổ chức.
-C. Trong kỳ thực tập
-•	Cách làm: Làm việc đúng giờ, tuân thủ nội quy công ty. Đặc biệt, hãy chủ động giữ liên lạc với giảng viên hướng dẫn tại trường (Academic Supervisor) để được hỗ trợ kịp thời nếu gặp khó khăn tại nơi làm việc.
-4. Lời khuyên "nằm lòng" để tối ưu hóa kỳ OJT
-•	Chọn công ty theo định hướng nghề nghiệp: Đừng chỉ chọn nơi nào "dễ". Hãy chọn nơi bạn có thể học được kỹ năng mình thiếu hoặc nơi bạn dự định làm việc sau khi ra trường.
-•	Xem OJT như một "phỏng vấn dài hạn": Nhiều sinh viên được nhận vào làm chính thức ngay sau khi kết thúc kỳ thực tập. Hãy thể hiện thái độ làm việc chuyên nghiệp, cầu thị và trách nhiệm.
-•	Ghi chép nhật ký công việc: Đừng đợi đến cuối kỳ mới ngồi viết báo cáo. Hãy ghi lại những gì mình học được, những vấn đề mình đã giải quyết mỗi tuần. Điều này giúp báo cáo thực tập của bạn trở nên sâu sắc và thuyết phục.
-•	Chủ động networking: Đừng chỉ ngồi làm việc một mình. Hãy kết nối với đồng nghiệp, người hướng dẫn (Mentor) tại công ty. Mối quan hệ trong kỳ thực tập là tài sản cực kỳ quý giá.
-5. Checklist kiểm tra nhanh
-•	[ ] Đã hoàn thành đủ tín chỉ điều kiện cho kỳ OJT chưa?
-•	[ ] CV/Portfolio đã được trau chuốt và phản ánh đúng năng lực hiện tại chưa?
-•	[ ] Đã nắm rõ các mốc deadline báo cáo thực tập (định kỳ) chưa?
-•	[ ] Đã có thông tin liên lạc của Giảng viên hướng dẫn tại trường chưa?
-Mẹo nhỏ: Trước khi bắt đầu, hãy tìm hiểu kỹ Rubric chấm điểm thực tập của trường. Bạn cần hiểu nhà trường đánh giá bạn dựa trên những tiêu chí nào (thái độ, kỹ năng, sản phẩm đầu ra...) để tập trung thể hiện đúng các điểm đó trong suốt kỳ thực tập.</t>
-  </si>
-  <si>
-    <t>phòng dịch vụ sinh viên</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Student Affairs là gì?
+Mẹo nhỏ: Hãy lập một file Excel cá nhân để tự tính toán điểm môn học theo thời gian thực (real-time). Khi biết rõ mình đang đứng ở mức nào, bạn sẽ biết cần dồn bao nhiêu sức lực cho bài thi cuối kỳ để đạt được mức điểm mong muốn (ví dụ: đạt điểm B hoặc A).</t>
+  </si>
+  <si>
+    <t>1. Student Affairs là gì?
 Student Affairs (Phòng Dịch vụ sinh viên - hay còn gọi là Phòng CTSV) là đơn vị đóng vai trò "người đồng hành" của sinh viên tại Đại học FPT. Nếu FAP là công cụ kỹ thuật, thì Student Affairs chính là bộ phận hỗ trợ trực tiếp các vấn đề về quyền lợi, đời sống, kỷ luật, hoạt động ngoại khóa và tinh thần của sinh viên. Đây là nơi bạn tìm đến khi gặp khó khăn không thuộc về chuyên môn học thuật đơn thuần.
 2. Các chức năng "Sống còn" tại Student Affairs
 Chức năng	Mục đích
@@ -660,38 +778,7 @@
 •	[ ] Đã chuẩn bị đầy đủ các giấy tờ, bằng chứng (nếu có) trước khi gặp cán bộ chưa?
 •	[ ] Đã xác định được "đúng người, đúng việc" (đúng bộ phận phụ trách vấn đề của mình) chưa?
 •	[ ] Đã có lịch hẹn hoặc thời gian làm việc của phòng chưa?
-Mẹo nhỏ: Hãy "kết thân" với thông tin của bộ phận Student Affairs ngay từ kỳ đầu tiên. Biết được ai là cán bộ quản lý khối lớp của mình, biết nơi nào để nộp đơn từ sẽ giúp bạn cực kỳ bình tĩnh khi gặp sự cố, thay vì chạy đôn chạy đáo khắp nơi để hỏi.
-</t>
-  </si>
-  <si>
-    <t>học phí</t>
-  </si>
-  <si>
-    <t>1. Tuition Fee là gì?
-Tuition Fee (Học phí) tại Đại học FPT là khoản chi phí sinh viên phải đóng để duy trì lộ trình học tập. ĐH FPT áp dụng mô hình thu học phí theo gói (tín chỉ) hoặc học kỳ, tùy thuộc vào hợp đồng đào tạo bạn đã ký lúc nhập học. Việc quản lý học phí chặt chẽ là điều kiện tiên quyết để bạn giữ trạng thái "Active" (đang học) trên hệ thống.
-2. Các khoản phí chính
-•	Học phí chính khóa: Tính theo tín chỉ hoặc mức cố định theo kỳ (tùy theo khóa và chương trình).
-•	Học phí tiếng Anh dự bị: Khoản phí bắt buộc nếu bạn chưa đủ điều kiện tiếng Anh đầu vào.
-•	Phí giáo trình: Thường đã bao gồm trong học phí hoặc được tính riêng tùy theo quy định của từng cơ sở.
-•	Phí môn học lại/học cải thiện: Phát sinh nếu bạn đăng ký Retake hoặc cải thiện điểm.
-3. Hướng dẫn thực hiện đóng học phí
-A. Tra cứu số tiền cần đóng
-•	Cách làm: Đăng nhập vào FAP -&gt; Chọn mục Financial -&gt; View tuition.
-•	Lưu ý: Hệ thống luôn cập nhật số dư, số tiền đã đóng và số tiền còn thiếu. Hãy kiểm tra định kỳ trước mỗi đợt hạn chót (Deadline).
-B. Quy trình thanh toán
-•	Cách làm: Thanh toán qua mã QR (trong FAP), chuyển khoản ngân hàng theo đúng Mã số sinh viên + Họ tên (theo quy định của từng cơ sở).
-•	Lưu ý: Sau khi chuyển khoản, hãy giữ lại biên lai/ảnh chụp giao dịch. Nếu sau 24-48h trạng thái trên FAP chưa cập nhật, hãy gửi biên lai đó cho Phòng Kế toán hoặc bộ phận hỗ trợ học phí.
-4. Lời khuyên "nằm lòng" để quản lý tài chính
-•	Luôn đóng sớm hơn Deadline: Đừng bao giờ để đến ngày cuối cùng mới đóng. Lỗi ngân hàng hoặc lỗi hệ thống vào giờ chót có thể khiến bạn bị trễ hạn, dẫn đến việc bị khóa quyền đăng ký môn học hoặc mất quyền thi.
-•	Lập kế hoạch tài chính: Nếu gia đình cần chuẩn bị tài chính, hãy chủ động xem trước mức học phí từng kỳ trong Hợp đồng đào tạo. Học phí tại FPT thường tăng nhẹ (tùy lộ trình) hoặc thay đổi dựa trên số tín chỉ bạn đăng ký, hãy dự phòng dư ra khoảng 5-10%.
-•	Tận dụng học bổng để giảm gánh nặng: Nếu GPA của bạn tốt, hãy săn các gói học bổng khuyến học để giảm bớt học phí. Đó là cách tốt nhất để "đầu tư" vào việc học.
-•	Liên hệ sớm nếu gặp khó khăn: Nếu gia đình gặp sự cố tài chính đột xuất, hãy chủ động viết đơn xin gia hạn học phí gửi lên Phòng Dịch vụ sinh viên trước ngày hết hạn. Đừng đợi đến khi bị khóa FAP mới xin, khả năng được duyệt sẽ thấp hơn rất nhiều.
-5. Checklist kiểm tra nhanh mỗi kỳ
-•	[ ] Đã check số tiền cần đóng trên FAP chưa?
-•	[ ] Đã nắm rõ hạn chót (Deadline) của đợt đóng học phí này chưa?
-•	[ ] Đã thanh toán và lưu lại ảnh biên lai chuyển khoản chưa?
-•	[ ] Trạng thái thanh toán trên FAP đã chuyển sang "Paid" (Đã thanh toán) chưa?
-Mẹo nhỏ: Hãy sử dụng tính năng "Reminder" trên điện thoại để đặt lịch nhắc đóng học phí trước deadline 3-5 ngày. Với sinh viên, việc bị khóa tài khoản chỉ vì quên đóng học phí là một trải nghiệm rất "đắt giá" và gây ảnh hưởng lớn đến tâm lý cũng như lộ trình học tập.</t>
+Mẹo nhỏ: Hãy "kết thân" với thông tin của bộ phận Student Affairs ngay từ kỳ đầu tiên. Biết được ai là cán bộ quản lý khối lớp của mình, biết nơi nào để nộp đơn từ sẽ giúp bạn cực kỳ bình tĩnh khi gặp sự cố, thay vì chạy đôn chạy đáo khắp nơi để hỏi.</t>
   </si>
   <si>
     <t>1. Email FPT là gì?
@@ -708,7 +795,7 @@
 •	Cách làm: Tải ứng dụng Outlook trên điện thoại. Đăng nhập bằng email FPT.
 •	Lưu ý: Hãy bật thông báo (push notifications) cho ứng dụng này. Việc nhận được thông báo thay đổi phòng học hoặc lịch thi ngay trên màn hình khóa điện thoại có thể cứu bạn khỏi những tình huống dở khóc dở cười.
 C. Quy tắc ứng xử khi gửi email
-•	Luôn có tiêu đề (Subject) rõ ràng: [Mã môn - Tên môn] - Nội dung cần hỏi.
+•	Luôn có tiêu đề (Subject) rõ ràng: [Họ và tên - MSSV] - [Mã môn - Tên môn] - Nội dung cần hỏi.
 •	Ghi rõ họ tên, mã số sinh viên, lớp ở cuối thư.
 •	Ngôn ngữ lịch sự, chuẩn mực.
 4. Lời khuyên "nằm lòng" để tối ưu hiệu quả
@@ -730,10 +817,10 @@
 Tại ĐH FPT, Final Grade không chỉ dựa vào điểm thi cuối kỳ mà là tổng hòa của nhiều thành phần:
 	Điểm thành phần: Các bài Assignment, Quiz, Mid-term, Presentation, Participation (thái độ tham gia lớp học).
 	Điểm Final Exam: Thường là kỳ thi bắt buộc tập trung. Lưu ý: Một số môn học có quy định điểm Final Exam phải đạt tối thiểu (ví dụ 4.0/10) mới được xét pass môn, bất kể điểm trung bình tổng kết có cao đến đâu.
-	Tổng hợp: Final Grade = ∑▒("Điểm từng cột" ×"Trọng số" ) .
+	Tổng hợp: Final Grade = ∑("Điểm từng cột" ×"Trọng số" ) .
 3. Hướng dẫn thực hiện và kiểm soát
 A. Theo dõi quá trình (Tracking)
-	Cách làm: Truy cập FAP -&gt; Grade -&gt; Academic Transcript.
+	Cách làm: Truy cập FAP -&gt; Reports -&gt; Academic Transcript.
 	Lưu ý: Mọi điểm thành phần phải được giảng viên cập nhật minh bạch trong quá trình học. Đừng để đến cuối kỳ mới kiểm tra.
 B. Quy trình phúc khảo (Review)
 	Cách làm: Khi Final Grade được công bố, nếu bạn thấy không khớp với kết quả tự tính, hãy liên hệ giảng viên hoặc Phòng Đào tạo (Academic Department) để xin phúc khảo theo quy trình chính thức.
@@ -749,9 +836,6 @@
 	[ ] Điểm hiển thị trên FAP có khớp với các bài đã được chấm không?
 	[ ] Bạn đã nắm rõ quy định về điểm thi Final tối thiểu chưa?
 Mẹo nhỏ: Hãy tự tạo một file "Dự báo điểm" (Grade Predictor). Sau mỗi bài kiểm tra, hãy cập nhật điểm vào đó. Việc biết chính xác mình đang ở ngưỡng nào (ví dụ: cần thêm bao nhiêu điểm để đạt mức B) sẽ giúp bạn điều chỉnh tâm lý và thời gian ôn tập cho bài Final Exam hiệu quả hơn rất nhiều.</t>
-  </si>
-  <si>
-    <t>Final Grade</t>
   </si>
   <si>
     <t>1. Course Schedule là gì?
@@ -781,12 +865,6 @@
 Mẹo nhỏ: Nếu bạn có các môn học cách nhau quá xa trong cùng một ngày (ví dụ: học sáng và tối), hãy tìm các bạn trong lớp có cùng lịch để cùng nhau "cắm chốt" tại thư viện hoặc quán cà phê gần trường. Việc có bạn đồng hành sẽ khiến những ngày "lịch dày" trở nên dễ thở hơn rất nhiều.</t>
   </si>
   <si>
-    <t>Course Schedule</t>
-  </si>
-  <si>
-    <t>IT Support</t>
-  </si>
-  <si>
     <t>1. IT Support là gì?
 IT Support tại Đại học FPT là bộ phận kỹ thuật phụ trách duy trì hạ tầng mạng, hệ thống phần mềm, và hỗ trợ các sự cố máy tính, tài khoản trong môi trường học đường. Đây là nơi bạn cần liên hệ khi gặp trục trặc về "công cụ" học tập (FAP, Wifi, Email, tài khoản học Online...).
 2. Các phạm vi hỗ trợ chính
@@ -798,7 +876,7 @@
 A. Quy trình báo lỗi (Ticket)
 Cách làm: Gửi email tới địa chỉ hỗ trợ kỹ thuật chính thức của cơ sở (thường được niêm yết trên bảng tin tại phòng Lab hoặc cuối trang FAP) hoặc trực tiếp đến quầy IT tại phòng Lab.
 Nội dung email cần có:
-Tiêu đề: [Hỗ trợ kỹ thuật] - [Mã số sinh viên] - [Vấn đề gặp phải].
+Tiêu đề: [Hỗ trợ kỹ thuật] - [Họ và tên] - [Mã số sinh viên] - [Vấn đề gặp phải].
 Nội dung: Mô tả chi tiết lỗi, kèm theo ảnh chụp màn hình (Screenshot) lỗi đó.
 Thông tin máy tính (nếu có): Tên máy đang sử dụng, vị trí phòng Lab.
 B. Xử lý sự cố Wifi/Mạng
@@ -814,91 +892,6 @@
 [ ] Lỗi này là do mạng (Wifi) hay do tài khoản (Login)?
 [ ] Đã gửi email báo lỗi hoặc đến quầy IT chưa?
 Mẹo nhỏ: Hãy lưu số điện thoại hoặc email của bộ phận IT cơ sở vào danh bạ điện thoại. Khi đang trong giờ thi hoặc giờ học mà gặp sự cố tài khoản, bạn sẽ cần liên hệ họ cực nhanh để không làm gián đoạn bài thi của mình!</t>
-  </si>
-  <si>
-    <t>1. Feedback là gì?
-Feedback tại Đại học FPT là hoạt động bắt buộc và mang tính chất định kỳ nhằm giúp sinh viên đánh giá năng lực, phương pháp giảng dạy và thái độ của giảng viên. Đây là kênh thông tin quan trọng nhất để nhà trường nâng cao chất lượng đào tạo. Việc hoàn thành Feedback là điều kiện bắt buộc để bạn có thể xem điểm tổng kết môn học (Final Grade) trên FAP.
-2. Các cột mốc Feedback cần lưu ý
-•	Feedback giữa kỳ (Mid-term Feedback): Thường diễn ra sau khoảng 5-7 tuần học. Mục đích là để giảng viên nắm bắt tâm lý sinh viên, từ đó điều chỉnh tốc độ hoặc phương pháp giảng dạy ngay trong kỳ học đó.
-•	Feedback cuối kỳ (End-term Feedback): Diễn ra trước khi kết thúc học kỳ. Đây là bản đánh giá tổng quát về toàn bộ khóa học.
-•	Lưu ý: Nếu bạn không hoàn thành Feedback đúng hạn, hệ thống FAP sẽ tạm khóa tính năng xem điểm của môn học đó.
-3. Hướng dẫn thực hiện Feedback
-A. Cách thực hiện
-•	Cách làm: Truy cập FAP -&gt; Feedback -&gt; Feedback for lecturers.
-•	Lựa chọn: Hệ thống sẽ liệt kê danh sách các môn học và giảng viên tương ứng. Bạn chọn môn cần thực hiện và trả lời các câu hỏi đánh giá theo thang điểm (thường từ 1-5 hoặc 1-7).
-B. Quy trình bảo mật
-•	Lưu ý: Mọi đánh giá của bạn là ẩn danh. Giảng viên chỉ nhận được kết quả tổng hợp (điểm trung bình và các góp ý chung), họ không thể biết đích danh sinh viên nào đã viết ý kiến gì.
-4. Lời khuyên "nằm lòng" để Feedback có giá trị
-•	Tính trung thực: Đây là quyền lợi của bạn. Nếu phương pháp dạy quá nhanh, bài giảng khó hiểu, hay cách chấm điểm chưa hợp lý, hãy thẳng thắn góp ý. Ý kiến của bạn là cơ sở để nhà trường yêu cầu giảng viên cải thiện.
-•	Góp ý cụ thể (Phần comment): Đừng chỉ đánh giá bằng các con số. Ở phần bình luận, hãy ghi rõ các ví dụ cụ thể (ví dụ: "Giảng viên cần nói to hơn", "Nên cho thêm bài tập thực hành", "Tốc độ dạy hơi nhanh ở chương 3"). Những góp ý chi tiết này rất có giá trị với giảng viên.
-•	Tâm thế xây dựng: Feedback không phải là công cụ để "trả đũa" cá nhân. Hãy đánh giá công tâm dựa trên chất lượng môn học và thái độ của giảng viên. Một Feedback mang tính xây dựng sẽ được nhà trường và giảng viên coi trọng hơn nhiều.
-•	Đừng để đến phút cuối: Hãy hoàn thành Feedback ngay khi có thông báo. Đừng đợi đến đúng ngày xem điểm mới vào làm, lúc đó hệ thống có thể bị quá tải.
-5. Checklist kiểm tra nhanh
-•	[ ] Đã nhận được thông báo thực hiện Feedback trên FAP chưa?
-•	[ ] Đã hoàn thành Feedback cho tất cả các môn học trong kỳ chưa?
-•	[ ] Các góp ý đã được viết một cách cụ thể, rõ ràng chưa?
-•	[ ] Đã kiểm tra lại trên FAP xem môn học đó đã hiện trạng thái "Completed" (đã hoàn thành) chưa?
-Mẹo nhỏ: Hãy dành riêng 15 phút mỗi kỳ để thực hiện Feedback một cách nghiêm túc. Hãy coi đây là cách bạn góp phần định hình chất lượng đào tạo tại FPT. Một sinh viên biết cách Feedback văn minh và cụ thể cũng chính là người đang rèn luyện kỹ năng đánh giá (critical thinking) rất tốt cho công việc sau này.</t>
-  </si>
-  <si>
-    <t>1. Student Management là gì?
-Student Management (Quản lý sinh viên) tại Đại học FPT không phải là một chức năng đơn lẻ mà là một hệ thống các quy định, quy trình và bộ phận chuyên trách nhằm quản lý toàn diện đời sống, học tập và tư cách sinh viên từ khi nhập học đến khi tốt nghiệp. Hệ thống này đảm bảo mọi sinh viên tuân thủ đúng Quy chế đào tạo và Student Handbook.
-2. Các nhóm vấn đề trọng yếu
-•	Hồ sơ sinh viên: Quản lý thông tin cá nhân, bằng cấp đầu vào, giấy tờ lưu trữ.
-•	Trạng thái sinh viên (Status): Quản lý tình trạng học tập (Active, Bảo lưu - Suspend, Thôi học - Drop out, Tốt nghiệp).
-•	Điểm rèn luyện: Đánh giá đạo đức, sự tham gia phong trào, đóng góp cộng đồng.
-•	Kỷ luật học đường: Xử lý các vi phạm về quy chế thi cử, thái độ với giảng viên, hay các quy định về trang phục/tác phong tại trường.
-3. Hướng dẫn thực hiện các tác vụ liên quan
-A. Thủ tục hành chính (Bảo lưu, Chuyển cơ sở, Nghỉ học)
-•	Cách làm: Truy cập FAP -&gt; Student Service -&gt; Submit Request. Điền form và chờ xác nhận từ phòng quản lý sinh viên.
-•	Lưu ý: Mọi yêu cầu liên quan đến trạng thái học tập đều yêu cầu bạn phải có lý do chính đáng và kèm minh chứng (ví dụ: giấy khám bệnh, quyết định điều động công tác...).
-B. Theo dõi điểm rèn luyện
-•	Cách làm: Kiểm tra định kỳ tại mục Student Life trên FAP.
-•	Lưu ý: Điểm rèn luyện thấp có thể ảnh hưởng đến cơ hội xét học bổng và xét tốt nghiệp.
-C. Cập nhật thông tin cá nhân
-•	Cách làm: Luôn đảm bảo email cá nhân, số điện thoại, và địa chỉ liên lạc trên FAP là mới nhất. Đây là nguồn thông tin chính để nhà trường liên hệ với gia đình bạn trong các tình huống khẩn cấp.
-4. Lời khuyên "nằm lòng" để quản lý bản thân tốt nhất
-•	Hiểu rõ "Student Handbook": Đây là "bộ luật" của trường. Mọi hành vi của bạn nếu vi phạm sẽ bị xử lý theo quy định trong này. Hãy đọc ít nhất 1 lần để biết "đường biên" cho phép của mình đến đâu.
-•	Chủ động cập nhật trạng thái: Nếu bạn cần bảo lưu (vì lý do cá nhân hoặc tài chính), hãy làm đơn càng sớm càng tốt. Việc tự ý nghỉ học mà không làm thủ tục bảo lưu sẽ khiến bạn bị tính "vắng không phép" và dẫn đến bị buộc thôi học (Drop out).
-•	Xây dựng "Hồ sơ sạch": Trong suốt quá trình học, tránh để xảy ra các lỗi kỷ luật. Một hồ sơ kỷ luật không chỉ ảnh hưởng đến kỳ học đó mà còn có thể gây khó khăn khi bạn xin xác nhận thực tập hoặc xin việc sau này (một số doanh nghiệp sẽ yêu cầu xem bảng điểm rèn luyện/kỷ luật).
-•	Giữ liên hệ với "người quản lý trực tiếp": Biết được cán bộ nào phụ trách khối lớp của mình (Block Manager) là vô cùng quan trọng. Hãy lưu thông tin liên lạc của họ để hỏi ngay khi có thắc mắc về hồ sơ.
-5. Checklist kiểm tra nhanh
-•	[ ] Thông tin cá nhân (SĐT, Email) trên FAP đã chính xác chưa?
-•	[ ] Đã kiểm tra điểm rèn luyện định kỳ chưa? (Đủ điều kiện xét tốt nghiệp không?)
-•	[ ] Có đang dự định thay đổi trạng thái học tập (bảo lưu, chuyển cơ sở) không? Nếu có, đã tìm hiểu kỹ quy trình trên FAP chưa?
-•	[ ] Đã đọc quy chế về kỷ luật học đường chưa?
-Mẹo nhỏ: Hãy tạo một thư mục riêng trên máy tính hoặc Google Drive để lưu tất cả các văn bản, giấy xác nhận, biên lai học phí mà bạn đã làm thủ tục. Khi nhà trường cần kiểm tra lại hồ sơ quản lý của bạn, bạn có thể xuất trình bằng chứng ngay lập tức mà không mất thời gian chờ đợi tra cứu từ hệ thống.</t>
-  </si>
-  <si>
-    <t>Student Management</t>
-  </si>
-  <si>
-    <t>1. Project là gì?
-Tại Đại học FPT, Project là học phần thực hành quan trọng, nơi sinh viên vận dụng kiến thức lý thuyết đã học trong một hoặc nhiều môn chuyên ngành để xây dựng một sản phẩm thực tế (phần mềm, ứng dụng, website, nghiên cứu...). Đây là "bài thi tổng hợp" thay thế cho các kỳ thi truyền thống, giúp sinh viên làm quen với cách làm việc nhóm và quy trình phát triển sản phẩm chuyên nghiệp.
-2. Các quy định "Sống còn"
-•	Hình thức: Thường là làm theo nhóm (từ 3-5 thành viên).
-•	Quy trình chuẩn: Sinh viên phải thực hiện theo đúng các giai đoạn: Requirement Analysis (Phân tích) -&gt; Design (Thiết kế) -&gt; Implementation (Lập trình) -&gt; Testing (Kiểm thử) -&gt; Documentation (Viết báo cáo).
-•	Deadline: Project thường có các cột mốc kiểm tra (Milestones/Reviews) định kỳ. Nếu không hoàn thành đúng tiến độ từng Milestone, nhóm sẽ bị đánh giá thấp hoặc thậm chí là "cấm thi" bảo vệ cuối kỳ.
-3. Hướng dẫn thực hiện chi tiết
-A. Xây dựng nhóm
-•	Cách làm: Tìm các thành viên có kỹ năng bổ trợ cho nhau (ví dụ: người giỏi code, người giỏi tài liệu, người giỏi trình bày).
-•	Lưu ý: "Chọn bạn mà chơi" trong Project là yếu tố quyết định 70% thành bại. Hãy chọn những thành viên có trách nhiệm và cùng mục tiêu điểm số.
-B. Quản lý công việc (Work Management)
-•	Cách làm: Sử dụng các công cụ quản lý dự án như Trello, Jira, hoặc GitHub Projects. Phải có bảng phân chia công việc (Task) rõ ràng cho từng thành viên.
-•	Lưu ý: Mọi công việc phải được ghi nhận (Track). Đừng làm việc theo kiểu "ai tiện thì làm", sẽ dẫn đến tình trạng tranh chấp hoặc đùn đẩy trách nhiệm khi gần đến ngày nộp bài.
-C. Bảo vệ Project
-•	Cách làm: Chuẩn bị slide trình bày (Presentation) thật chuyên nghiệp, nắm vững kiến thức sản phẩm và có khả năng trả lời phản biện (Q&amp;A) từ giảng viên.
-4. Lời khuyên "nằm lòng" để đạt điểm cao
-•	Bám sát Rubric: Giảng viên chấm điểm dựa trên bộ tiêu chí (Rubric) đã ban hành. Hãy đọc kỹ nó trước khi bắt đầu. Nếu Rubric nhấn mạnh vào "Tính năng mới", hãy tập trung làm tính năng đó trước thay vì chỉ chăm chút giao diện.
-•	Documentation quan trọng không kém Code: Đừng coi nhẹ bài báo cáo (Documentation). Nhiều nhóm làm sản phẩm cực tốt nhưng báo cáo sơ sài dẫn đến điểm tổng kết rất thấp. Hãy trình bày tài liệu theo đúng form chuẩn của trường.
-•	Tận dụng giảng viên hướng dẫn (Mentor): Đừng đợi đến khi sản phẩm "tắt thở" mới hỏi giảng viên. Hãy chủ động cập nhật tiến độ (Meeting định kỳ) với Mentor để được chỉnh hướng ngay khi đi sai đường.
-•	Giải quyết xung đột nội bộ sớm: Nếu nhóm có thành viên không làm việc, hãy giải quyết ngay từ Milestone đầu tiên. Đừng đợi đến cuối kỳ mới báo cáo với giảng viên, lúc đó việc tách nhóm hay thay đổi nhân sự sẽ rất khó khăn.
-5. Checklist kiểm tra nhanh
-•	[ ] Đã hiểu rõ yêu cầu (Requirements) của đề bài chưa?
-•	[ ] Đã phân chia Task cho từng thành viên trên công cụ quản lý chưa?
-•	[ ] Đã có lịch họp nhóm định kỳ hàng tuần chưa?
-•	[ ] Đã nắm rõ các mốc Review/Milestone chưa?
-Mẹo nhỏ: Hãy dành thời gian làm Demo sớm. Sản phẩm chạy được sớm dù chỉ là bản thô (Prototype) sẽ giúp bạn nhận được phản hồi từ giảng viên ngay từ đầu. Điều này giúp bạn tránh phải "đập đi xây lại" toàn bộ dự án vào tuần cuối cùng trước ngày nộp bài.</t>
   </si>
 </sst>
 </file>
@@ -1275,10 +1268,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1592,7 +1581,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
@@ -1600,39 +1589,39 @@
         <v>23</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
@@ -1640,23 +1629,23 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="360" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="388.8" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="374.4" x14ac:dyDescent="0.3">
@@ -1664,23 +1653,23 @@
         <v>13</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
@@ -1688,31 +1677,31 @@
         <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="360" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="360" x14ac:dyDescent="0.3">
@@ -1720,15 +1709,15 @@
         <v>14</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="388.8" x14ac:dyDescent="0.3">
@@ -1736,7 +1725,7 @@
         <v>6</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>